<commit_message>
Day 5: Implemented Runner file and modified Step Definition, Page Objects and added cookies manager
</commit_message>
<xml_diff>
--- a/Automation_Testing/NoBroker_BDD_Framework/src/test/resources/TestData/PackersAndMovers.xlsx
+++ b/Automation_Testing/NoBroker_BDD_Framework/src/test/resources/TestData/PackersAndMovers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/51585ef60b1564a3/Desktop/QA/NoBroker_QA/Automation_Testing/NoBroker_BDD_Framework/src/test/resources/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{D964A728-037E-40A6-8650-801FF0DCF2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C92A7ECE-7E52-4A1D-8566-C154D7885838}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{D964A728-037E-40A6-8650-801FF0DCF2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A3B84E8-5A62-467E-A9C7-17D423304F99}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="12090" xr2:uid="{76AF94B6-2AED-4649-AD67-24C9B9E00330}"/>
+    <workbookView xWindow="3220" yWindow="3220" windowWidth="14400" windowHeight="8710" xr2:uid="{76AF94B6-2AED-4649-AD67-24C9B9E00330}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
   <si>
     <t>TC_ID</t>
   </si>
@@ -50,18 +50,12 @@
     <t>item</t>
   </si>
   <si>
+    <t>type</t>
+  </si>
+  <si>
     <t>category</t>
   </si>
   <si>
-    <t>TC_01</t>
-  </si>
-  <si>
-    <t>TC_02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cox Town </t>
-  </si>
-  <si>
     <t>Yelahanka</t>
   </si>
   <si>
@@ -71,7 +65,7 @@
     <t>Koramangala</t>
   </si>
   <si>
-    <t>Bedroom</t>
+    <t>Bed</t>
   </si>
   <si>
     <t>searchItem</t>
@@ -80,12 +74,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t>BedKing Size Bed - With Storage</t>
-  </si>
-  <si>
-    <t>TC_03</t>
-  </si>
-  <si>
     <t>koramangala</t>
   </si>
   <si>
@@ -101,7 +89,22 @@
     <t>Cap</t>
   </si>
   <si>
-    <t>TC_04</t>
+    <t>TC01</t>
+  </si>
+  <si>
+    <t>TC02</t>
+  </si>
+  <si>
+    <t>TC03</t>
+  </si>
+  <si>
+    <t>TC04</t>
+  </si>
+  <si>
+    <t>Bedrooms</t>
+  </si>
+  <si>
+    <t>Diwan Cum Bed</t>
   </si>
 </sst>
 </file>
@@ -167,6 +170,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -486,16 +493,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AEED651-14F9-4715-B937-35079820F2F7}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.08984375" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="26.54296875" customWidth="1"/>
-    <col min="6" max="6" width="28.453125" customWidth="1"/>
+    <col min="5" max="5" width="9.08984375" customWidth="1"/>
+    <col min="7" max="7" width="28.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,87 +514,108 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="36.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
+      <c r="G5" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>